<commit_message>
pushing to B dog, whoops should have done this earlier
</commit_message>
<xml_diff>
--- a/Input_Files/Peirson_IcePhenoDates_AVG_20250120.xlsx
+++ b/Input_Files/Peirson_IcePhenoDates_AVG_20250120.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Gagers/Documents/Thesis and Lab/Ice Phenology Project/Ice_Pheno/Input_Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaga3666/repos/Ice_Pheno/Input_Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746F8E74-ED23-244F-B13A-7D8AE3B227CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB31D08-A157-9045-B6F5-A67080866956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="740" windowWidth="23840" windowHeight="15260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="5">
   <si>
     <t>Ice_On_Peirson</t>
   </si>
@@ -29,6 +29,12 @@
   </si>
   <si>
     <t>waterYear</t>
+  </si>
+  <si>
+    <t>siteID</t>
+  </si>
+  <si>
+    <t>LOC</t>
   </si>
 </sst>
 </file>
@@ -385,102 +391,129 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="3" width="20.6640625" style="2" customWidth="1"/>
+    <col min="3" max="4" width="20.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
         <v>2017</v>
       </c>
-      <c r="B2" s="2">
+      <c r="C2" s="2">
         <v>42649</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>42929</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
         <v>2018</v>
       </c>
-      <c r="B3" s="2">
+      <c r="C3" s="2">
         <v>43035</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3" s="2">
         <v>43241</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
         <v>2019</v>
       </c>
-      <c r="B4" s="2">
+      <c r="C4" s="2">
         <v>43417</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D4" s="2">
         <v>43641</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
         <v>2020</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
         <v>2021</v>
       </c>
-      <c r="B6" s="2">
+      <c r="C6" s="2">
         <v>44121</v>
       </c>
-      <c r="C6" s="2">
+      <c r="D6" s="2">
         <v>44361</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
         <v>2022</v>
       </c>
-      <c r="B7" s="2">
+      <c r="C7" s="2">
         <v>44481</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D7" s="2">
         <v>44720</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
         <v>2023</v>
       </c>
-      <c r="B8" s="2">
+      <c r="C8" s="2">
         <v>44850</v>
       </c>
-      <c r="C8" s="2">
+      <c r="D8" s="2">
         <v>45091</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
         <v>2024</v>
       </c>
-      <c r="B9" s="2">
+      <c r="C9" s="2">
         <v>45227</v>
       </c>
-      <c r="C9" s="2">
+      <c r="D9" s="2">
         <v>45453</v>
       </c>
     </row>

</xml_diff>